<commit_message>
update timeline for Tyler
</commit_message>
<xml_diff>
--- a/Market Makers Project Timeline.xlsx
+++ b/Market Makers Project Timeline.xlsx
@@ -1,17 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tyler_hyposvu\UW\ECE554\ECE554_Capstone\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0656789-0FC9-411B-ABF7-DDACA83C2979}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="Sheet1" sheetId="1" r:id="rId5"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="52">
   <si>
     <t>Project Part</t>
   </si>
@@ -75,9 +84,6 @@
     <t xml:space="preserve">Tyler Chen </t>
   </si>
   <si>
-    <t>Order Books (Full level book</t>
-  </si>
-  <si>
     <t>Trading Logic (Volatility)</t>
   </si>
   <si>
@@ -151,31 +157,89 @@
   </si>
   <si>
     <t>Poster &amp; Report Work</t>
+  </si>
+  <si>
+    <t>Before Spring Break</t>
+  </si>
+  <si>
+    <t>3/26 - 4/8</t>
+  </si>
+  <si>
+    <t>4/9 - 4/15</t>
+  </si>
+  <si>
+    <t>4/16 - 4/22</t>
+  </si>
+  <si>
+    <t>4/23 - 4/29</t>
+  </si>
+  <si>
+    <t>Order Price Book Finished and Tested (2 stage pipeline).
+Full Level Book Finished
+Cache is 90% finished, waiting for Refill Engine to support the insert part</t>
+  </si>
+  <si>
+    <t>Refilling Engine with Epoch finsihed.
+Full FLB is tested in simulation.
+Designed an integration test for orderbook.
+Orderbook top module tested in both simulation and integration (7 stage pipeline).</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="m/d"/>
   </numFmts>
-  <fonts count="3">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
-      <sz val="10.0"/>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -184,7 +248,7 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -200,48 +264,53 @@
     </fill>
   </fills>
   <borders count="1">
-    <border/>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+  <cellXfs count="10">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="3" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -431,24 +500,29 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:J27"/>
+  <sheetFormatPr defaultColWidth="12.59765625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="26.25"/>
-    <col customWidth="1" min="2" max="2" width="38.13"/>
-    <col customWidth="1" min="3" max="3" width="17.75"/>
-    <col customWidth="1" min="4" max="4" width="17.25"/>
-    <col customWidth="1" min="5" max="5" width="96.13"/>
+    <col min="1" max="1" width="26.265625" customWidth="1"/>
+    <col min="2" max="2" width="38.1328125" customWidth="1"/>
+    <col min="3" max="3" width="17.73046875" customWidth="1"/>
+    <col min="4" max="4" width="17.265625" customWidth="1"/>
+    <col min="5" max="5" width="96.1328125" customWidth="1"/>
+    <col min="6" max="6" width="31.9296875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="29.73046875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A1" s="1"/>
       <c r="B1" s="1" t="s">
         <v>0</v>
@@ -462,8 +536,23 @@
       <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2">
+      <c r="F1" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="G1" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="H1" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="I1" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="J1" s="7" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
@@ -477,7 +566,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A3" s="2"/>
       <c r="B3" s="2" t="s">
         <v>8</v>
@@ -492,7 +581,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A4" s="2"/>
       <c r="B4" s="2" t="s">
         <v>12</v>
@@ -504,7 +593,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A5" s="2"/>
       <c r="B5" s="2" t="s">
         <v>14</v>
@@ -519,7 +608,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A6" s="2"/>
       <c r="B6" s="2" t="s">
         <v>17</v>
@@ -531,7 +620,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" spans="1:10" ht="102" x14ac:dyDescent="0.35">
       <c r="A7" s="2"/>
       <c r="B7" s="2" t="s">
         <v>18</v>
@@ -542,201 +631,195 @@
       <c r="D7" s="3" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="8">
+      <c r="F7" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="G7" s="9" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" ht="12.75" x14ac:dyDescent="0.35">
       <c r="A8" s="2"/>
       <c r="B8" s="2" t="s">
         <v>20</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="D8" s="3" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A9" s="2"/>
       <c r="B9" s="2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="D9" s="3" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A10" s="2"/>
       <c r="B10" s="2" t="s">
         <v>23</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="D10" s="3" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="11">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A11" s="2"/>
       <c r="B11" s="2" t="s">
         <v>24</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="D11" s="3" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="12">
+        <v>25</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A12" s="2"/>
       <c r="B12" s="2" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="D12" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="E12" s="2" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="13">
+        <v>15</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A13" s="2"/>
       <c r="B13" s="2" t="s">
         <v>28</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D13" s="3" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="14">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A14" s="2"/>
       <c r="B14" s="2" t="s">
         <v>29</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="D14" s="3" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="2"/>
-      <c r="B15" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="C15" s="2" t="s">
+    <row r="16" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A16" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="D15" s="3" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="1" t="s">
+      <c r="B16" s="2" t="s">
         <v>32</v>
       </c>
+      <c r="C16" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D16" s="4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B17" s="2" t="s">
         <v>33</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D17" s="4" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="B18" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A21" s="1"/>
+      <c r="B21" s="1"/>
+    </row>
+    <row r="22" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A22" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="C18" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="D18" s="3" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="1"/>
-      <c r="B22" s="1"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="1" t="s">
+      <c r="B22" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C22" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="B23" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C23" s="1" t="s">
+      <c r="D22" s="1"/>
+      <c r="E22" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="D23" s="1"/>
-      <c r="E23" s="1" t="s">
+    </row>
+    <row r="23" spans="1:5" ht="12.75" x14ac:dyDescent="0.35">
+      <c r="A23" s="2"/>
+      <c r="B23" s="2" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="2"/>
+      <c r="C23" s="5">
+        <v>46124</v>
+      </c>
+      <c r="E23" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" ht="12.75" x14ac:dyDescent="0.35">
       <c r="B24" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C24" s="5">
-        <v>46124.0</v>
+        <v>46128</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="25">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" ht="12.75" x14ac:dyDescent="0.35">
       <c r="B25" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C25" s="5">
-        <v>46128.0</v>
+        <v>46128</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="26">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" ht="12.75" x14ac:dyDescent="0.35">
       <c r="B26" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C26" s="5">
-        <v>46128.0</v>
-      </c>
-      <c r="E26" s="2" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="27">
+        <v>46133</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" ht="12.75" x14ac:dyDescent="0.35">
       <c r="B27" s="2" t="s">
         <v>44</v>
       </c>
       <c r="C27" s="5">
-        <v>46133.0</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="B28" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="C28" s="5">
-        <v>46140.0</v>
+        <v>46140</v>
       </c>
     </row>
   </sheetData>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Finished top level and top level tb
Updated spreadsheet and made top level + tb. Top level tb needs more tests
</commit_message>
<xml_diff>
--- a/Market Makers Project Timeline.xlsx
+++ b/Market Makers Project Timeline.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tyler_hyposvu\UW\ECE554\ECE554_Capstone\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DanielJL\Documents\GitHub\ECE554_Capstone\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0656789-0FC9-411B-ABF7-DDACA83C2979}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98D900A9-4757-469F-9430-2E92AF1FEA02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="59">
   <si>
     <t>Project Part</t>
   </si>
@@ -100,9 +100,6 @@
   </si>
   <si>
     <t>Daniel Lei, Will Strong</t>
-  </si>
-  <si>
-    <t>Just need to put everything together and verify successful logic (profits) once complete</t>
   </si>
   <si>
     <t xml:space="preserve">Risk Management </t>
@@ -183,6 +180,30 @@
 Full FLB is tested in simulation.
 Designed an integration test for orderbook.
 Orderbook top module tested in both simulation and integration (7 stage pipeline).</t>
+  </si>
+  <si>
+    <t>Created but not tested</t>
+  </si>
+  <si>
+    <t>Created and tested in simulation</t>
+  </si>
+  <si>
+    <t>Tested and simulated</t>
+  </si>
+  <si>
+    <t>All submodules are put together and has testbench to verify mid-price, reservation based on inventory , spread based on inventory, and time of day behavior . Can be labelled complete since the core functionality works but want to improve coverage so a few additional test cases will be created to target edge cases.</t>
+  </si>
+  <si>
+    <t>Waiting for submodules to be completed</t>
+  </si>
+  <si>
+    <t>Full top level created and connected with submodules. Testbench created and tests core functionaltiy but want to test extra edge cases</t>
+  </si>
+  <si>
+    <t xml:space="preserve">New volatility module follows EWMA and is finished and tested </t>
+  </si>
+  <si>
+    <t xml:space="preserve">New volatility module was created but not tested </t>
   </si>
 </sst>
 </file>
@@ -275,7 +296,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -290,6 +311,12 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -511,18 +538,18 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:J27"/>
-  <sheetFormatPr defaultColWidth="12.59765625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="12.5546875" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="26.265625" customWidth="1"/>
-    <col min="2" max="2" width="38.1328125" customWidth="1"/>
-    <col min="3" max="3" width="17.73046875" customWidth="1"/>
-    <col min="4" max="4" width="17.265625" customWidth="1"/>
-    <col min="5" max="5" width="96.1328125" customWidth="1"/>
-    <col min="6" max="6" width="31.9296875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="29.73046875" customWidth="1"/>
+    <col min="1" max="1" width="26.21875" customWidth="1"/>
+    <col min="2" max="2" width="38.109375" customWidth="1"/>
+    <col min="3" max="3" width="17.77734375" customWidth="1"/>
+    <col min="4" max="4" width="17.21875" customWidth="1"/>
+    <col min="5" max="5" width="96.109375" customWidth="1"/>
+    <col min="6" max="6" width="31.88671875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="29.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1"/>
       <c r="B1" s="1" t="s">
         <v>0</v>
@@ -537,22 +564,22 @@
         <v>3</v>
       </c>
       <c r="F1" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="G1" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="G1" s="7" t="s">
+      <c r="H1" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="H1" s="7" t="s">
+      <c r="I1" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="I1" s="7" t="s">
+      <c r="J1" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="J1" s="7" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+    </row>
+    <row r="2" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
@@ -566,7 +593,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:10" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A3" s="2"/>
       <c r="B3" s="2" t="s">
         <v>8</v>
@@ -581,7 +608,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:10" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A4" s="2"/>
       <c r="B4" s="2" t="s">
         <v>12</v>
@@ -593,7 +620,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:10" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A5" s="2"/>
       <c r="B5" s="2" t="s">
         <v>14</v>
@@ -608,7 +635,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:10" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A6" s="2"/>
       <c r="B6" s="2" t="s">
         <v>17</v>
@@ -620,7 +647,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="102" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:10" ht="105.6" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="2" t="s">
         <v>18</v>
@@ -632,13 +659,13 @@
         <v>7</v>
       </c>
       <c r="F7" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="G7" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="G7" s="9" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" ht="12.75" x14ac:dyDescent="0.35">
+    </row>
+    <row r="8" spans="1:10" ht="26.4" x14ac:dyDescent="0.25">
       <c r="A8" s="2"/>
       <c r="B8" s="2" t="s">
         <v>20</v>
@@ -649,8 +676,14 @@
       <c r="D8" s="3" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="F8" s="10" t="s">
+        <v>58</v>
+      </c>
+      <c r="G8" s="11" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A9" s="2"/>
       <c r="B9" s="2" t="s">
         <v>22</v>
@@ -661,8 +694,10 @@
       <c r="D9" s="3" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="F9" s="11"/>
+      <c r="G9" s="11"/>
+    </row>
+    <row r="10" spans="1:10" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A10" s="2"/>
       <c r="B10" s="2" t="s">
         <v>23</v>
@@ -673,8 +708,12 @@
       <c r="D10" s="3" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="F10" s="11"/>
+      <c r="G10" s="11" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" ht="66" x14ac:dyDescent="0.25">
       <c r="A11" s="2"/>
       <c r="B11" s="2" t="s">
         <v>24</v>
@@ -685,14 +724,20 @@
       <c r="D11" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="E11" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="E11" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="F11" s="11" t="s">
+        <v>55</v>
+      </c>
+      <c r="G11" s="11" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A12" s="2"/>
       <c r="B12" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>15</v>
@@ -700,11 +745,13 @@
       <c r="D12" s="3" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="F12" s="11"/>
+      <c r="G12" s="11"/>
+    </row>
+    <row r="13" spans="1:10" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A13" s="2"/>
       <c r="B13" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C13" s="2" t="s">
         <v>13</v>
@@ -712,25 +759,33 @@
       <c r="D13" s="3" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="F13" s="11"/>
+      <c r="G13" s="11"/>
+    </row>
+    <row r="14" spans="1:10" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A14" s="2"/>
       <c r="B14" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C14" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="C14" s="2" t="s">
+      <c r="D14" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="F14" s="10" t="s">
+        <v>51</v>
+      </c>
+      <c r="G14" s="11" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="D14" s="3" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A16" s="1" t="s">
+      <c r="B16" s="2" t="s">
         <v>31</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>32</v>
       </c>
       <c r="C16" s="2" t="s">
         <v>15</v>
@@ -739,9 +794,9 @@
         <v>10</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:5" ht="13.2" x14ac:dyDescent="0.25">
       <c r="B17" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C17" s="2" t="s">
         <v>19</v>
@@ -750,70 +805,70 @@
         <v>7</v>
       </c>
     </row>
-    <row r="21" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="1"/>
       <c r="B21" s="1"/>
     </row>
-    <row r="22" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B22" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D22" s="1"/>
       <c r="E22" s="1" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" ht="12.75" x14ac:dyDescent="0.35">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A23" s="2"/>
       <c r="B23" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C23" s="5">
         <v>46124</v>
       </c>
       <c r="E23" s="2" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="B24" s="2" t="s">
         <v>38</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" ht="12.75" x14ac:dyDescent="0.35">
-      <c r="B24" s="2" t="s">
-        <v>39</v>
       </c>
       <c r="C24" s="5">
         <v>46128</v>
       </c>
       <c r="E24" s="2" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="B25" s="2" t="s">
         <v>40</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" ht="12.75" x14ac:dyDescent="0.35">
-      <c r="B25" s="2" t="s">
-        <v>41</v>
       </c>
       <c r="C25" s="5">
         <v>46128</v>
       </c>
       <c r="E25" s="2" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="B26" s="2" t="s">
         <v>42</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" ht="12.75" x14ac:dyDescent="0.35">
-      <c r="B26" s="2" t="s">
-        <v>43</v>
       </c>
       <c r="C26" s="5">
         <v>46133</v>
       </c>
     </row>
-    <row r="27" spans="1:5" ht="12.75" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:5" ht="13.2" x14ac:dyDescent="0.25">
       <c r="B27" s="2" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C27" s="5">
         <v>46140</v>

</xml_diff>

<commit_message>
corrected the integration status: have not include parser yet
</commit_message>
<xml_diff>
--- a/Market Makers Project Timeline.xlsx
+++ b/Market Makers Project Timeline.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\edwar\OneDrive\Documents\Coding\ECE 554\ECE554_Capstone\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tyler_hyposvu\UW\ECE554\ECE554_Capstone\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{743FF27F-4A41-410F-9F68-D8D6EDEC6C9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A593B17D-AEDE-471F-988F-8D47DD08E3DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -184,9 +184,6 @@
     <t/>
   </si>
   <si>
-    <t>Parser -&gt; OrderBooks tested on board</t>
-  </si>
-  <si>
     <t xml:space="preserve">Future Goals &amp; Roadmap: </t>
   </si>
   <si>
@@ -240,6 +237,9 @@
   </si>
   <si>
     <t>Created hps_tcp_reciever.py and verified packet communcation between laptop and FPGA. Also created tcp_packet_reciever.v but unable to program the board succesfully.</t>
+  </si>
+  <si>
+    <t>OrderBooks tested on board</t>
   </si>
 </sst>
 </file>
@@ -702,20 +702,20 @@
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:J27"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="26.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="38.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.7109375" style="13" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="96.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="31.85546875" style="9" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="29.7109375" style="9" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="29.42578125" bestFit="1" customWidth="1"/>
-    <col min="9" max="10" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.265625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="38.1328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.73046875" style="13" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.265625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="96.1328125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="31.86328125" style="9" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="29.73046875" style="9" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="29.3984375" bestFit="1" customWidth="1"/>
+    <col min="9" max="10" width="13.59765625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A1" s="1"/>
       <c r="B1" s="1" t="s">
         <v>0</v>
@@ -745,7 +745,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="60" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" ht="42.75" x14ac:dyDescent="0.45">
       <c r="A2" s="1" t="s">
         <v>9</v>
       </c>
@@ -759,11 +759,11 @@
         <v>12</v>
       </c>
       <c r="F2" s="16" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G2"/>
     </row>
-    <row r="3" spans="1:10" ht="105" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" ht="85.5" x14ac:dyDescent="0.45">
       <c r="A3" s="6"/>
       <c r="B3" s="6" t="s">
         <v>13</v>
@@ -775,16 +775,16 @@
         <v>15</v>
       </c>
       <c r="E3" s="17" t="s">
+        <v>67</v>
+      </c>
+      <c r="F3" s="18" t="s">
         <v>68</v>
       </c>
-      <c r="F3" s="18" t="s">
+      <c r="G3" s="19" t="s">
         <v>69</v>
       </c>
-      <c r="G3" s="19" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" ht="39" x14ac:dyDescent="0.25">
+    </row>
+    <row r="4" spans="1:10" ht="39" x14ac:dyDescent="0.45">
       <c r="A4" s="6"/>
       <c r="B4" s="6" t="s">
         <v>16</v>
@@ -796,10 +796,10 @@
         <v>12</v>
       </c>
       <c r="F4" s="15" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A5" s="6"/>
       <c r="B5" s="6" t="s">
         <v>18</v>
@@ -820,7 +820,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A6" s="6"/>
       <c r="B6" s="6" t="s">
         <v>23</v>
@@ -835,7 +835,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="102.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:10" ht="102.75" x14ac:dyDescent="0.45">
       <c r="A7" s="6"/>
       <c r="B7" s="6" t="s">
         <v>25</v>
@@ -853,7 +853,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="8" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:10" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A8" s="6"/>
       <c r="B8" s="6" t="s">
         <v>29</v>
@@ -871,7 +871,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="9" spans="1:10" ht="26.25" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:10" ht="26.25" x14ac:dyDescent="0.45">
       <c r="A9" s="6"/>
       <c r="B9" s="6" t="s">
         <v>33</v>
@@ -884,10 +884,10 @@
       </c>
       <c r="F9" s="12"/>
       <c r="G9" s="15" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A10" s="6"/>
       <c r="B10" s="6" t="s">
         <v>34</v>
@@ -903,7 +903,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="75" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:10" ht="57" x14ac:dyDescent="0.45">
       <c r="A11" s="6"/>
       <c r="B11" s="6" t="s">
         <v>36</v>
@@ -924,7 +924,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A12" s="6"/>
       <c r="B12" s="6" t="s">
         <v>41</v>
@@ -940,7 +940,7 @@
       </c>
       <c r="G12" s="12"/>
     </row>
-    <row r="13" spans="1:10" ht="39" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:10" ht="39" x14ac:dyDescent="0.45">
       <c r="A13" s="6"/>
       <c r="B13" s="6" t="s">
         <v>43</v>
@@ -953,10 +953,10 @@
       </c>
       <c r="F13" s="12"/>
       <c r="G13" s="15" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A14" s="6"/>
       <c r="B14" s="6" t="s">
         <v>44</v>
@@ -974,7 +974,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="16" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:10" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A16" s="1" t="s">
         <v>48</v>
       </c>
@@ -994,9 +994,9 @@
         <v>51</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.45">
       <c r="B17" s="6" t="s">
-        <v>52</v>
+        <v>70</v>
       </c>
       <c r="C17" s="7" t="s">
         <v>26</v>
@@ -1005,70 +1005,70 @@
         <v>12</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A21" s="1"/>
       <c r="B21" s="1"/>
     </row>
-    <row r="22" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A22" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B22" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D22" s="1"/>
       <c r="E22" s="1" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A23" s="6"/>
       <c r="B23" s="6" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C23" s="7">
         <v>46124</v>
       </c>
       <c r="E23" s="6" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="B24" s="6" t="s">
         <v>57</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B24" s="6" t="s">
-        <v>58</v>
       </c>
       <c r="C24" s="7">
         <v>46128</v>
       </c>
       <c r="E24" s="6" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="B25" s="6" t="s">
         <v>59</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B25" s="6" t="s">
-        <v>60</v>
       </c>
       <c r="C25" s="7">
         <v>46128</v>
       </c>
       <c r="E25" s="6" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="B26" s="6" t="s">
         <v>61</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B26" s="6" t="s">
-        <v>62</v>
       </c>
       <c r="C26" s="7">
         <v>46133</v>
       </c>
     </row>
-    <row r="27" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B27" s="6" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C27" s="7">
         <v>46140</v>

</xml_diff>

<commit_message>
Updated trading logic test benches, finished up trading logic top level, and updated timeline
</commit_message>
<xml_diff>
--- a/Market Makers Project Timeline.xlsx
+++ b/Market Makers Project Timeline.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wills\ECE554\ECE554_Capstone\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DanielJL\Documents\GitHub\ECE554_Capstone\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{157A8342-A696-454B-B6C6-8B04C55F9C4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7C15E0A-ACFB-47DE-8E5F-B0AB7C30C45C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="14020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="82">
   <si>
     <t>Project Part</t>
   </si>
@@ -261,6 +261,18 @@
   </si>
   <si>
     <t>Simulation of the market and our FPGA trading logic to work out ideal parameters for risk and liquidity</t>
+  </si>
+  <si>
+    <t>Added more tests and fully tested</t>
+  </si>
+  <si>
+    <t>Trading Logic (Time)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tested and works in relation to market open duration </t>
+  </si>
+  <si>
+    <t>Full level testbench complete follows, Avallenda Stoikov algorithm</t>
   </si>
 </sst>
 </file>
@@ -379,7 +391,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -436,9 +448,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -756,21 +765,21 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:J27"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:J28"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="26.26953125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="38.08984375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.7265625" style="13" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.26953125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="96.08984375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="31.81640625" style="9" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="29.7265625" style="9" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="29.36328125" bestFit="1" customWidth="1"/>
-    <col min="9" max="10" width="13.6328125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.21875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="38.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.77734375" style="13" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.21875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="96.109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="31.77734375" style="9" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="29.77734375" style="9" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="29.33203125" bestFit="1" customWidth="1"/>
+    <col min="9" max="10" width="13.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" s="1"/>
       <c r="B1" s="1" t="s">
         <v>0</v>
@@ -800,7 +809,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>9</v>
       </c>
@@ -818,7 +827,7 @@
       </c>
       <c r="G2"/>
     </row>
-    <row r="3" spans="1:10" ht="87" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:10" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A3" s="6"/>
       <c r="B3" s="6" t="s">
         <v>13</v>
@@ -842,7 +851,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="38.5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:10" ht="40.200000000000003" x14ac:dyDescent="0.3">
       <c r="A4" s="6"/>
       <c r="B4" s="6" t="s">
         <v>16</v>
@@ -857,7 +866,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A5" s="6"/>
       <c r="B5" s="6" t="s">
         <v>18</v>
@@ -878,7 +887,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" s="6"/>
       <c r="B6" s="6" t="s">
         <v>23</v>
@@ -893,7 +902,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="88.5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:10" ht="106.2" x14ac:dyDescent="0.3">
       <c r="A7" s="6"/>
       <c r="B7" s="6" t="s">
         <v>25</v>
@@ -914,7 +923,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="8" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A8" s="6"/>
       <c r="B8" s="6" t="s">
         <v>29</v>
@@ -931,8 +940,11 @@
       <c r="G8" s="12" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="9" spans="1:10" ht="26" x14ac:dyDescent="0.35">
+      <c r="H8" s="9" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" ht="27" x14ac:dyDescent="0.3">
       <c r="A9" s="6"/>
       <c r="B9" s="6" t="s">
         <v>33</v>
@@ -948,10 +960,10 @@
         <v>64</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A10" s="6"/>
       <c r="B10" s="6" t="s">
-        <v>34</v>
+        <v>79</v>
       </c>
       <c r="C10" s="7" t="s">
         <v>30</v>
@@ -960,211 +972,233 @@
         <v>12</v>
       </c>
       <c r="F10" s="12"/>
-      <c r="G10" s="12" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" ht="72.5" x14ac:dyDescent="0.35">
+      <c r="G10" s="15" t="s">
+        <v>46</v>
+      </c>
+      <c r="H10" s="9" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A11" s="6"/>
       <c r="B11" s="6" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="D11" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="E11" s="11" t="s">
-        <v>38</v>
-      </c>
-      <c r="F11" s="12" t="s">
-        <v>39</v>
-      </c>
+        <v>30</v>
+      </c>
+      <c r="D11" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="F11" s="12"/>
       <c r="G11" s="12" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" ht="72" x14ac:dyDescent="0.3">
       <c r="A12" s="6"/>
       <c r="B12" s="6" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="D12" s="8" t="s">
-        <v>12</v>
+        <v>37</v>
+      </c>
+      <c r="D12" s="19" t="s">
+        <v>12</v>
+      </c>
+      <c r="E12" s="11" t="s">
+        <v>38</v>
       </c>
       <c r="F12" s="12" t="s">
-        <v>42</v>
-      </c>
-      <c r="G12" s="12"/>
-    </row>
-    <row r="13" spans="1:10" ht="38.5" x14ac:dyDescent="0.35">
+        <v>39</v>
+      </c>
+      <c r="G12" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="H12" s="9" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A13" s="6"/>
       <c r="B13" s="6" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="D13" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="F13" s="12"/>
-      <c r="G13" s="15" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="F13" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="G13" s="12"/>
+    </row>
+    <row r="14" spans="1:10" ht="40.200000000000003" x14ac:dyDescent="0.3">
       <c r="A14" s="6"/>
       <c r="B14" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="C14" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="D14" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="F14" s="12"/>
+      <c r="G14" s="15" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A15" s="6"/>
+      <c r="B15" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="C14" s="7" t="s">
+      <c r="C15" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="D14" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="F14" s="11" t="s">
+      <c r="D15" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="F15" s="11" t="s">
         <v>46</v>
       </c>
-      <c r="G14" s="12" t="s">
+      <c r="G15" s="12" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="15" spans="1:10" s="9" customFormat="1" ht="58" x14ac:dyDescent="0.35">
-      <c r="B15" s="21" t="s">
+    <row r="16" spans="1:10" s="9" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="B16" s="11" t="s">
         <v>76</v>
       </c>
-      <c r="C15" s="22" t="s">
+      <c r="C16" s="21" t="s">
         <v>17</v>
       </c>
-      <c r="D15" s="23" t="s">
-        <v>12</v>
-      </c>
-      <c r="H15" s="9" t="s">
+      <c r="D16" s="22" t="s">
+        <v>12</v>
+      </c>
+      <c r="H16" s="9" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="H16" s="14" t="s">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="H17" s="14" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="17" spans="1:7" ht="29" x14ac:dyDescent="0.35">
-      <c r="A17" s="1" t="s">
+    <row r="18" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A18" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="B17" s="6" t="s">
+      <c r="B18" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="C17" s="7" t="s">
+      <c r="C18" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="D17" s="10" t="s">
+      <c r="D18" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="G17" s="9" t="s">
+      <c r="G18" s="9" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="B18" s="6" t="s">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="B19" s="6" t="s">
         <v>69</v>
       </c>
-      <c r="C18" s="7" t="s">
+      <c r="C19" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="D18" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="E18" t="s">
+      <c r="D19" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="E19" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="B19" s="6" t="s">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="B20" s="6" t="s">
         <v>72</v>
       </c>
-      <c r="C19" s="13" t="s">
+      <c r="C20" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="D19" s="20" t="s">
-        <v>12</v>
-      </c>
-      <c r="E19" t="s">
+      <c r="D20" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="E20" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A21" s="1"/>
-      <c r="B21" s="1"/>
-    </row>
-    <row r="22" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A22" s="1" t="s">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A22" s="1"/>
+      <c r="B22" s="1"/>
+    </row>
+    <row r="23" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="B22" s="1" t="s">
+      <c r="B23" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C22" s="2" t="s">
+      <c r="C23" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="D22" s="1"/>
-      <c r="E22" s="1" t="s">
+      <c r="D23" s="1"/>
+      <c r="E23" s="1" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="23" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="6"/>
-      <c r="B23" s="6" t="s">
+    <row r="24" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="6"/>
+      <c r="B24" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="C23" s="7">
+      <c r="C24" s="7">
         <v>46124</v>
       </c>
-      <c r="E23" s="6" t="s">
+      <c r="E24" s="6" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="24" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B24" s="6" t="s">
+    <row r="25" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B25" s="6" t="s">
         <v>57</v>
-      </c>
-      <c r="C24" s="7">
-        <v>46128</v>
-      </c>
-      <c r="E24" s="6" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B25" s="6" t="s">
-        <v>59</v>
       </c>
       <c r="C25" s="7">
         <v>46128</v>
       </c>
       <c r="E25" s="6" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B26" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="C26" s="7">
+        <v>46128</v>
+      </c>
+      <c r="E26" s="6" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="26" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B26" s="6" t="s">
+    <row r="27" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B27" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="C26" s="7">
+      <c r="C27" s="7">
         <v>46133</v>
       </c>
     </row>
-    <row r="27" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B27" s="6" t="s">
+    <row r="28" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B28" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="C27" s="7">
+      <c r="C28" s="7">
         <v>46140</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Market Makers Project Timeline.xlsx
</commit_message>
<xml_diff>
--- a/Market Makers Project Timeline.xlsx
+++ b/Market Makers Project Timeline.xlsx
@@ -1,20 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion rupBuild="9303" lowestEdited="5" lastEdited="5" appName="xl"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29822"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\edwar\OneDrive\Documents\Coding\ECE 554\ECE554_Capstone\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC691A93-EEFF-4190-8BF4-4796FE6E3D08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="0"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet r:id="rId1" sheetId="1" name="Sheet1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr fullCalcOnLoad="1"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="238" uniqueCount="89">
   <si>
     <t>Project Part</t>
   </si>
@@ -73,9 +79,6 @@
   </si>
   <si>
     <t>Created hps_tcp_reciever.py and verified packet communcation between laptop and FPGA. Also created tcp_packet_reciever.v but unable to program the board succesfully.</t>
-  </si>
-  <si>
-    <t>Fixed issues connecting HPS and FPGA logic. Ethernet Input complete. Ethernet Output complete. Need to merge with ITCH translator.</t>
   </si>
   <si>
     <t>Parser</t>
@@ -278,23 +281,49 @@
     <t>Demo team (software showing all stocks &amp; info)</t>
   </si>
   <si>
-    <t xml:space="preserve">Execution tracker in python should have most information on inventory, profits, and trades ready, just needs to make graphs and look pretty. </t>
-  </si>
-  <si>
     <t>Final Improvements, bug fixes, and internal demo</t>
   </si>
   <si>
     <t>Poster &amp; Report Work</t>
+  </si>
+  <si>
+    <t>Fixed issues connecting HPS and FPGA logic. Ethernet Input complete. Ethernet Output complete. Ethenet Connected to both parser and translator</t>
+  </si>
+  <si>
+    <r>
+      <t>Execution tracker in python should have most information on inventory, profits, and trades ready, just needs to make graphs and look pretty.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> Facing issues when connecting Parser and Orderbook.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> Hope to fix by the end of 4/16.</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve"> Facing issues when connecting Parser and Orderbook.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="m/d"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -333,6 +362,19 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FFFF0000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -343,17 +385,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF00ff00"/>
+        <fgColor rgb="FF00FF00"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF66ff33"/>
+        <fgColor rgb="FF66FF33"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFffff00"/>
+        <fgColor rgb="FFFFFF00"/>
       </patternFill>
     </fill>
   </fills>
@@ -374,16 +416,16 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="FFc6c6c6"/>
+        <color rgb="FFC6C6C6"/>
       </left>
       <right style="thin">
-        <color rgb="FFc6c6c6"/>
+        <color rgb="FFC6C6C6"/>
       </right>
       <top style="thin">
-        <color rgb="FFc6c6c6"/>
+        <color rgb="FFC6C6C6"/>
       </top>
       <bottom style="thin">
-        <color rgb="FFc6c6c6"/>
+        <color rgb="FFC6C6C6"/>
       </bottom>
       <diagonal/>
     </border>
@@ -391,95 +433,84 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+  <cellXfs count="23">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general" wrapText="1"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="4" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="5" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="4" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" builtinId="0" name="Normal"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
-    <ext uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14ac:slicerStyles xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" defaultSlicerStyle="SlicerStyleLight1"/>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -490,10 +521,10 @@
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:sysClr lastClr="000000" val="windowText"/>
+        <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr lastClr="FFFFFF" val="window"/>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="000000"/>
@@ -531,71 +562,71 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
-        <a:font typeface="맑은 고딕" script="Hang"/>
-        <a:font typeface="宋体" script="Hans"/>
-        <a:font typeface="新細明體" script="Hant"/>
-        <a:font typeface="Times New Roman" script="Arab"/>
-        <a:font typeface="Times New Roman" script="Hebr"/>
-        <a:font typeface="Tahoma" script="Thai"/>
-        <a:font typeface="Nyala" script="Ethi"/>
-        <a:font typeface="Vrinda" script="Beng"/>
-        <a:font typeface="Shruti" script="Gujr"/>
-        <a:font typeface="MoolBoran" script="Khmr"/>
-        <a:font typeface="Tunga" script="Knda"/>
-        <a:font typeface="Raavi" script="Guru"/>
-        <a:font typeface="Euphemia" script="Cans"/>
-        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
-        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
-        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
-        <a:font typeface="MV Boli" script="Thaa"/>
-        <a:font typeface="Mangal" script="Deva"/>
-        <a:font typeface="Gautami" script="Telu"/>
-        <a:font typeface="Latha" script="Taml"/>
-        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
-        <a:font typeface="Kalinga" script="Orya"/>
-        <a:font typeface="Kartika" script="Mlym"/>
-        <a:font typeface="DokChampa" script="Laoo"/>
-        <a:font typeface="Iskoola Pota" script="Sinh"/>
-        <a:font typeface="Mongolian Baiti" script="Mong"/>
-        <a:font typeface="Times New Roman" script="Viet"/>
-        <a:font typeface="Microsoft Uighur" script="Uigh"/>
-        <a:font typeface="Sylfaen" script="Geor"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
-        <a:font typeface="맑은 고딕" script="Hang"/>
-        <a:font typeface="宋体" script="Hans"/>
-        <a:font typeface="新細明體" script="Hant"/>
-        <a:font typeface="Arial" script="Arab"/>
-        <a:font typeface="Arial" script="Hebr"/>
-        <a:font typeface="Tahoma" script="Thai"/>
-        <a:font typeface="Nyala" script="Ethi"/>
-        <a:font typeface="Vrinda" script="Beng"/>
-        <a:font typeface="Shruti" script="Gujr"/>
-        <a:font typeface="DaunPenh" script="Khmr"/>
-        <a:font typeface="Tunga" script="Knda"/>
-        <a:font typeface="Raavi" script="Guru"/>
-        <a:font typeface="Euphemia" script="Cans"/>
-        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
-        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
-        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
-        <a:font typeface="MV Boli" script="Thaa"/>
-        <a:font typeface="Mangal" script="Deva"/>
-        <a:font typeface="Gautami" script="Telu"/>
-        <a:font typeface="Latha" script="Taml"/>
-        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
-        <a:font typeface="Kalinga" script="Orya"/>
-        <a:font typeface="Kartika" script="Mlym"/>
-        <a:font typeface="DokChampa" script="Laoo"/>
-        <a:font typeface="Iskoola Pota" script="Sinh"/>
-        <a:font typeface="Mongolian Baiti" script="Mong"/>
-        <a:font typeface="Arial" script="Viet"/>
-        <a:font typeface="Microsoft Uighur" script="Uigh"/>
-        <a:font typeface="Sylfaen" script="Geor"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -623,7 +654,7 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin scaled="1" ang="16200000"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
@@ -646,11 +677,11 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin scaled="1" ang="16200000"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="9525">
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr">
               <a:shade val="9500"/>
@@ -659,13 +690,13 @@
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="25400">
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="38100">
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -675,7 +706,7 @@
       <a:effectStyleLst>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="38000"/>
               </a:srgbClr>
@@ -684,7 +715,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -693,7 +724,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -701,10 +732,10 @@
           </a:effectLst>
           <a:scene3d>
             <a:camera prst="orthographicFront">
-              <a:rot rev="0" lon="0" lat="0"/>
+              <a:rot lat="0" lon="0" rev="0"/>
             </a:camera>
-            <a:lightRig dir="t" rig="threePt">
-              <a:rot rev="1200000" lon="0" lat="0"/>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
             </a:lightRig>
           </a:scene3d>
           <a:sp3d>
@@ -769,26 +800,26 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:J28"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="23" width="26.290714285714284" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="24" width="38.14785714285715" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="25" width="17.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="23" width="17.290714285714284" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="23" width="96.14785714285713" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="26" width="31.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="26" width="29.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="26" width="29.290714285714284" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="23" width="22.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="23" width="13.719285714285713" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" width="26.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="38.140625" style="17" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.7109375" style="18" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="96.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="31.7109375" style="10" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="29.7109375" style="10" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="29.28515625" style="10" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="22.85546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
+    <row r="1" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1"/>
       <c r="B1" s="1" t="s">
         <v>0</v>
@@ -818,7 +849,7 @@
         <v>8</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="44.25">
+    <row r="2" spans="1:10" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>9</v>
       </c>
@@ -831,16 +862,11 @@
       <c r="D2" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="E2" s="9"/>
-      <c r="F2" s="10" t="s">
+      <c r="F2" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="G2" s="11"/>
-      <c r="H2" s="11"/>
-      <c r="I2" s="9"/>
-      <c r="J2" s="9"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="83.25">
+    </row>
+    <row r="3" spans="1:10" ht="83.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="6"/>
       <c r="B3" s="6" t="s">
         <v>14</v>
@@ -848,529 +874,403 @@
       <c r="C3" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="D3" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="E3" s="13" t="s">
+      <c r="D3" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="E3" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="F3" s="13" t="s">
+      <c r="F3" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="G3" s="10" t="s">
+      <c r="G3" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="H3" s="10" t="s">
-        <v>19</v>
-      </c>
-      <c r="I3" s="9"/>
-      <c r="J3" s="9"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="39">
+      <c r="H3" s="9" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" ht="39" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="6"/>
       <c r="B4" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="C4" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="D4" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="F4" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="D4" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="E4" s="9"/>
-      <c r="F4" s="14" t="s">
-        <v>22</v>
-      </c>
-      <c r="G4" s="11"/>
-      <c r="H4" s="11"/>
-      <c r="I4" s="9"/>
-      <c r="J4" s="9"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="31.5">
+    </row>
+    <row r="5" spans="1:10" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="6"/>
       <c r="B5" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="C5" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="C5" s="7" t="s">
+      <c r="D5" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="E5" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="D5" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="E5" s="6" t="s">
+      <c r="F5" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="F5" s="10" t="s">
+      <c r="G5" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="G5" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="H5" s="11"/>
-      <c r="I5" s="9"/>
-      <c r="J5" s="9"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
+    </row>
+    <row r="6" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="6"/>
       <c r="B6" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="D6" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="G6" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="C6" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="D6" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="E6" s="9"/>
-      <c r="F6" s="11"/>
-      <c r="G6" s="10" t="s">
+      <c r="H6" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="H6" s="11" t="s">
-        <v>30</v>
-      </c>
-      <c r="I6" s="9"/>
-      <c r="J6" s="9"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="94.5">
+    </row>
+    <row r="7" spans="1:10" ht="94.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="6"/>
       <c r="B7" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="C7" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="C7" s="7" t="s">
+      <c r="D7" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="E7" s="22" t="s">
+        <v>88</v>
+      </c>
+      <c r="F7" s="13" t="s">
         <v>32</v>
       </c>
-      <c r="D7" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="E7" s="9"/>
-      <c r="F7" s="14" t="s">
+      <c r="G7" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="G7" s="14" t="s">
+      <c r="H7" s="13" t="s">
         <v>34</v>
       </c>
-      <c r="H7" s="14" t="s">
-        <v>35</v>
-      </c>
-      <c r="I7" s="9"/>
-      <c r="J7" s="9"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="47.25">
+    </row>
+    <row r="8" spans="1:10" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="6"/>
       <c r="B8" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="C8" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="C8" s="7" t="s">
+      <c r="D8" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="F8" s="13" t="s">
         <v>37</v>
       </c>
-      <c r="D8" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="E8" s="9"/>
-      <c r="F8" s="14" t="s">
+      <c r="G8" s="14" t="s">
         <v>38</v>
       </c>
-      <c r="G8" s="15" t="s">
+      <c r="H8" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="H8" s="10" t="s">
-        <v>40</v>
-      </c>
-      <c r="I8" s="9"/>
-      <c r="J8" s="9"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="27.75">
+    </row>
+    <row r="9" spans="1:10" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="6"/>
       <c r="B9" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="C9" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D9" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="F9" s="14"/>
+      <c r="G9" s="13" t="s">
         <v>41</v>
       </c>
-      <c r="C9" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="D9" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="E9" s="9"/>
-      <c r="F9" s="15"/>
-      <c r="G9" s="14" t="s">
-        <v>42</v>
-      </c>
-      <c r="H9" s="11"/>
-      <c r="I9" s="9"/>
-      <c r="J9" s="9"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="31.5">
+    </row>
+    <row r="10" spans="1:10" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="6"/>
       <c r="B10" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="C10" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="D10" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="F10" s="14"/>
+      <c r="G10" s="13" t="s">
         <v>43</v>
       </c>
-      <c r="C10" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="D10" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="E10" s="9"/>
-      <c r="F10" s="15"/>
-      <c r="G10" s="14" t="s">
+      <c r="H10" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="H10" s="10" t="s">
-        <v>45</v>
-      </c>
-      <c r="I10" s="9"/>
-      <c r="J10" s="9"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="19.5">
+    </row>
+    <row r="11" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="6"/>
       <c r="B11" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="C11" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="D11" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="F11" s="14"/>
+      <c r="G11" s="14" t="s">
         <v>46</v>
       </c>
-      <c r="C11" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="D11" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="E11" s="9"/>
-      <c r="F11" s="15"/>
-      <c r="G11" s="15" t="s">
-        <v>47</v>
-      </c>
-      <c r="H11" s="11"/>
-      <c r="I11" s="9"/>
-      <c r="J11" s="9"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="75">
+    </row>
+    <row r="12" spans="1:10" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="6"/>
       <c r="B12" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="C12" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="C12" s="7" t="s">
+      <c r="D12" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="E12" s="13" t="s">
         <v>49</v>
       </c>
-      <c r="D12" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="E12" s="14" t="s">
+      <c r="F12" s="14" t="s">
         <v>50</v>
       </c>
-      <c r="F12" s="15" t="s">
+      <c r="G12" s="14" t="s">
         <v>51</v>
       </c>
-      <c r="G12" s="15" t="s">
+      <c r="H12" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="H12" s="10" t="s">
-        <v>53</v>
-      </c>
-      <c r="I12" s="9"/>
-      <c r="J12" s="9"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="19.5">
+    </row>
+    <row r="13" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="6"/>
       <c r="B13" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="C13" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="D13" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="F13" s="14" t="s">
         <v>54</v>
       </c>
-      <c r="C13" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="D13" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="E13" s="9"/>
-      <c r="F13" s="15" t="s">
+      <c r="G13" s="14"/>
+      <c r="H13" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="G13" s="15"/>
-      <c r="H13" s="11" t="s">
-        <v>56</v>
-      </c>
-      <c r="I13" s="9"/>
-      <c r="J13" s="9"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="39">
+    </row>
+    <row r="14" spans="1:10" ht="39" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="6"/>
       <c r="B14" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="C14" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D14" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="F14" s="14"/>
+      <c r="G14" s="13" t="s">
         <v>57</v>
       </c>
-      <c r="C14" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="D14" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="E14" s="9"/>
-      <c r="F14" s="15"/>
-      <c r="G14" s="14" t="s">
-        <v>58</v>
-      </c>
-      <c r="H14" s="11"/>
-      <c r="I14" s="9"/>
-      <c r="J14" s="9"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="19.5">
+    </row>
+    <row r="15" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="6"/>
       <c r="B15" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="C15" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="C15" s="7" t="s">
+      <c r="D15" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="F15" s="13" t="s">
+        <v>43</v>
+      </c>
+      <c r="G15" s="14" t="s">
         <v>60</v>
       </c>
-      <c r="D15" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="E15" s="9"/>
-      <c r="F15" s="14" t="s">
-        <v>44</v>
-      </c>
-      <c r="G15" s="15" t="s">
+    </row>
+    <row r="16" spans="1:10" s="10" customFormat="1" ht="57.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B16" s="13" t="s">
         <v>61</v>
       </c>
-      <c r="H15" s="11"/>
-      <c r="I15" s="9"/>
-      <c r="J15" s="9"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="57.75" customFormat="1" s="16">
-      <c r="A16" s="11"/>
-      <c r="B16" s="14" t="s">
+      <c r="C16" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="D16" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="H16" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="C16" s="17" t="s">
-        <v>21</v>
-      </c>
-      <c r="D16" s="18" t="s">
-        <v>12</v>
-      </c>
-      <c r="E16" s="11"/>
-      <c r="F16" s="11"/>
-      <c r="G16" s="11"/>
-      <c r="H16" s="10" t="s">
+    </row>
+    <row r="17" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="18" spans="1:9" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="I16" s="11"/>
-      <c r="J16" s="11"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="18.75">
-      <c r="A17" s="9"/>
-      <c r="B17" s="19"/>
-      <c r="C17" s="20"/>
-      <c r="D17" s="9"/>
-      <c r="E17" s="9"/>
-      <c r="F17" s="11"/>
-      <c r="G17" s="11"/>
-      <c r="H17" s="11"/>
-      <c r="I17" s="9"/>
-      <c r="J17" s="9"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="31.5">
-      <c r="A18" s="1" t="s">
+      <c r="B18" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="B18" s="6" t="s">
+      <c r="C18" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="D18" s="19" t="s">
+        <v>12</v>
+      </c>
+      <c r="G18" s="9" t="s">
         <v>65</v>
       </c>
-      <c r="C18" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="D18" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="E18" s="9"/>
-      <c r="F18" s="11"/>
-      <c r="G18" s="10" t="s">
+      <c r="H18" s="10" t="s">
         <v>66</v>
       </c>
-      <c r="H18" s="11" t="s">
+    </row>
+    <row r="19" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B19" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="I18" s="9"/>
-      <c r="J18" s="9"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="18.75">
-      <c r="A19" s="9"/>
-      <c r="B19" s="6" t="s">
+      <c r="C19" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="D19" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="E19" t="s">
         <v>68</v>
       </c>
-      <c r="C19" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="D19" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="E19" s="9" t="s">
+    </row>
+    <row r="20" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B20" s="6" t="s">
         <v>69</v>
       </c>
-      <c r="F19" s="11"/>
-      <c r="G19" s="11"/>
-      <c r="H19" s="11"/>
-      <c r="I19" s="9"/>
-      <c r="J19" s="9"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="18.75">
-      <c r="A20" s="9"/>
-      <c r="B20" s="6" t="s">
+      <c r="C20" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="D20" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="E20" t="s">
         <v>70</v>
       </c>
-      <c r="C20" s="22" t="s">
-        <v>32</v>
-      </c>
-      <c r="D20" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="E20" s="9" t="s">
+    </row>
+    <row r="21" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B21" s="17" t="s">
         <v>71</v>
       </c>
-      <c r="F20" s="11"/>
-      <c r="G20" s="11"/>
-      <c r="H20" s="11"/>
-      <c r="I20" s="9"/>
-      <c r="J20" s="9"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="18.75">
-      <c r="A21" s="9"/>
-      <c r="B21" s="19" t="s">
+      <c r="C21" s="18" t="s">
+        <v>23</v>
+      </c>
+      <c r="D21" t="s">
         <v>72</v>
       </c>
-      <c r="C21" s="20" t="s">
-        <v>24</v>
-      </c>
-      <c r="D21" s="9" t="s">
+      <c r="E21" t="s">
         <v>73</v>
       </c>
-      <c r="E21" s="9" t="s">
+      <c r="H21" s="10" t="s">
         <v>74</v>
       </c>
-      <c r="F21" s="11"/>
-      <c r="G21" s="11"/>
-      <c r="H21" s="11" t="s">
+      <c r="I21" t="s">
         <v>75</v>
       </c>
-      <c r="I21" s="9" t="s">
-        <v>76</v>
-      </c>
-      <c r="J21" s="9"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="18.75">
+    </row>
+    <row r="22" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="1"/>
       <c r="B22" s="1"/>
-      <c r="C22" s="20"/>
-      <c r="D22" s="9"/>
-      <c r="E22" s="9"/>
-      <c r="F22" s="11"/>
-      <c r="G22" s="11"/>
-      <c r="H22" s="11"/>
-      <c r="I22" s="9"/>
-      <c r="J22" s="9"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="18.75">
+    </row>
+    <row r="23" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B23" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D23" s="1"/>
       <c r="E23" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="F23" s="11"/>
-      <c r="G23" s="11"/>
-      <c r="H23" s="11"/>
-      <c r="I23" s="9"/>
-      <c r="J23" s="9"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="18.75">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="6"/>
       <c r="B24" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C24" s="7">
         <v>46124</v>
       </c>
-      <c r="D24" s="9"/>
       <c r="E24" s="6" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B25" s="6" t="s">
         <v>81</v>
-      </c>
-      <c r="F24" s="11"/>
-      <c r="G24" s="11"/>
-      <c r="H24" s="11"/>
-      <c r="I24" s="9"/>
-      <c r="J24" s="9"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="18.75">
-      <c r="A25" s="9"/>
-      <c r="B25" s="6" t="s">
-        <v>82</v>
       </c>
       <c r="C25" s="7">
         <v>46128</v>
       </c>
-      <c r="D25" s="9"/>
       <c r="E25" s="6" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" ht="50.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B26" s="6" t="s">
         <v>83</v>
-      </c>
-      <c r="F25" s="11"/>
-      <c r="G25" s="11"/>
-      <c r="H25" s="11"/>
-      <c r="I25" s="9"/>
-      <c r="J25" s="9"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="18.75">
-      <c r="A26" s="9"/>
-      <c r="B26" s="6" t="s">
-        <v>84</v>
       </c>
       <c r="C26" s="7">
         <v>46128</v>
       </c>
-      <c r="D26" s="9"/>
-      <c r="E26" s="6" t="s">
-        <v>85</v>
-      </c>
-      <c r="F26" s="11"/>
-      <c r="G26" s="11"/>
-      <c r="H26" s="11"/>
-      <c r="I26" s="9"/>
-      <c r="J26" s="9"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="27" customHeight="1" ht="18.75">
-      <c r="A27" s="9"/>
+      <c r="E26" s="21" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B27" s="6" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C27" s="7">
         <v>46133</v>
       </c>
-      <c r="D27" s="9"/>
-      <c r="E27" s="9"/>
-      <c r="F27" s="11"/>
-      <c r="G27" s="11"/>
-      <c r="H27" s="11"/>
-      <c r="I27" s="9"/>
-      <c r="J27" s="9"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="28" customHeight="1" ht="18.75">
-      <c r="A28" s="9"/>
+    </row>
+    <row r="28" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B28" s="6" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="C28" s="7">
         <v>46140</v>
       </c>
-      <c r="D28" s="9"/>
-      <c r="E28" s="9"/>
-      <c r="F28" s="11"/>
-      <c r="G28" s="11"/>
-      <c r="H28" s="11"/>
-      <c r="I28" s="9"/>
-      <c r="J28" s="9"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>